<commit_message>
Commit for Part 1
</commit_message>
<xml_diff>
--- a/Template_Part1_FILLED.xlsx
+++ b/Template_Part1_FILLED.xlsx
@@ -668,10 +668,10 @@
         <v>41670</v>
       </c>
       <c r="B2" s="16" t="n">
-        <v>-0.0287515686902544</v>
+        <v>-0.0292131277885951</v>
       </c>
       <c r="C2" s="17" t="n">
-        <v>-0.0435349935811963</v>
+        <v>-0.040489473451515</v>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
@@ -679,10 +679,10 @@
         </is>
       </c>
       <c r="F2" s="6" t="n">
-        <v>0.0794583733751737</v>
+        <v>0.0830195627376546</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>0.0670820558878524</v>
+        <v>0.0665507513182344</v>
       </c>
     </row>
     <row r="3">
@@ -690,10 +690,10 @@
         <v>41698</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0520933741461129</v>
+        <v>0.0443765407033162</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.019246991751624</v>
+        <v>0.0233194369943782</v>
       </c>
       <c r="E3" s="22" t="inlineStr">
         <is>
@@ -701,10 +701,10 @@
         </is>
       </c>
       <c r="F3" s="23" t="n">
-        <v>0.1154979005218071</v>
+        <v>0.1091921422059808</v>
       </c>
       <c r="G3" s="24" t="n">
-        <v>0.1291407141705315</v>
+        <v>0.1317393262428307</v>
       </c>
     </row>
     <row r="4">
@@ -712,10 +712,10 @@
         <v>41729</v>
       </c>
       <c r="B4" t="n">
-        <v>0.0171999188269799</v>
+        <v>0.0156953122327677</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.0026683714969575</v>
+        <v>0.0033717666371136</v>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
@@ -723,10 +723,10 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.6149194364167639</v>
+        <v>0.6724500627210289</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.4715005344785024</v>
+        <v>0.4610036347267343</v>
       </c>
     </row>
     <row r="5">
@@ -734,10 +734,10 @@
         <v>41759</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.0138280133872863</v>
+        <v>-0.0109291001904266</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.0068666427142612</v>
+        <v>-0.008777486381004</v>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
@@ -745,10 +745,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>-0.1242717964152482</v>
+        <v>-0.07849270332025569</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>-0.1075897946467893</v>
+        <v>-0.114422511974802</v>
       </c>
     </row>
     <row r="6">
@@ -756,10 +756,10 @@
         <v>41789</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0551363227448278</v>
+        <v>0.0549309396087019</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.0303178144934912</v>
+        <v>0.0305939730513512</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
@@ -767,10 +767,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.09832976236810401</v>
+        <v>0.1045673974044797</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.130681155663674</v>
+        <v>0.1329161675884338</v>
       </c>
     </row>
     <row r="7">
@@ -778,10 +778,10 @@
         <v>41820</v>
       </c>
       <c r="B7" t="n">
-        <v>0.0464646570539367</v>
+        <v>0.0482913607494455</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.0321672383779624</v>
+        <v>0.0336665196602827</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -789,10 +789,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.503057314399208</v>
+        <v>1.603967844856272</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>1.179584958580808</v>
+        <v>1.166597869346414</v>
       </c>
     </row>
     <row r="8">
@@ -800,10 +800,10 @@
         <v>41851</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0145399272475348</v>
+        <v>0.0142016332347468</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.0218518833323933</v>
+        <v>0.0168510014099256</v>
       </c>
       <c r="E8" s="9" t="n">
         <v>41791</v>
@@ -815,10 +815,10 @@
         <v>41880</v>
       </c>
       <c r="B9" s="18" t="n">
-        <v>0.0186444934104972</v>
+        <v>0.017697700494654</v>
       </c>
       <c r="C9" s="19" t="n">
-        <v>-0.0118456577284512</v>
+        <v>-0.0096844626509714</v>
       </c>
       <c r="E9" s="9" t="n">
         <v>41821</v>
@@ -830,10 +830,10 @@
         <v>41912</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.0283711875282875</v>
+        <v>-0.0263433169339023</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.0364315926541183</v>
+        <v>-0.0360519572703029</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>41852</v>
@@ -845,10 +845,10 @@
         <v>41943</v>
       </c>
       <c r="B11" t="n">
-        <v>0.0273074749854677</v>
+        <v>0.0193420059184127</v>
       </c>
       <c r="C11" t="n">
-        <v>0.008401628532876701</v>
+        <v>0.005930134348938</v>
       </c>
       <c r="E11" s="9" t="n">
         <v>41883</v>
@@ -867,10 +867,10 @@
         <v>42004</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.0177158807715862</v>
+        <v>-0.0194757840624766</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.0139599903273446</v>
+        <v>-0.0122061598634387</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>41944</v>
@@ -882,10 +882,10 @@
         <v>42034</v>
       </c>
       <c r="B14" t="n">
-        <v>0.0605192801397153</v>
+        <v>0.065019885756992</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0187933362315639</v>
+        <v>0.0158680652851171</v>
       </c>
       <c r="E14" s="9" t="n">
         <v>41974</v>
@@ -897,10 +897,10 @@
         <v>42062</v>
       </c>
       <c r="B15" t="n">
-        <v>0.0033634523149509</v>
+        <v>0.0019627321956429</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0482112925890249</v>
+        <v>0.0494236236252841</v>
       </c>
       <c r="E15" s="9" t="n">
         <v>42005</v>
@@ -912,10 +912,10 @@
         <v>42094</v>
       </c>
       <c r="B16" t="n">
-        <v>0.0068195056624802</v>
+        <v>0.008957117096824899</v>
       </c>
       <c r="C16" t="n">
-        <v>0.008504657454357301</v>
+        <v>0.0012029148529209</v>
       </c>
       <c r="E16" s="9" t="n">
         <v>42036</v>
@@ -927,10 +927,10 @@
         <v>42124</v>
       </c>
       <c r="B17" t="n">
-        <v>0.030106299647049</v>
+        <v>0.0391241918545165</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0434155333491115</v>
+        <v>0.038556978762711</v>
       </c>
       <c r="E17" s="9" t="n">
         <v>42064</v>
@@ -942,10 +942,10 @@
         <v>42153</v>
       </c>
       <c r="B18" t="n">
-        <v>0.005014841359876</v>
+        <v>0.0094834150813734</v>
       </c>
       <c r="C18" t="n">
-        <v>-0.0004879380389377</v>
+        <v>-0.0015612515201332</v>
       </c>
       <c r="E18" s="9" t="n">
         <v>42095</v>
@@ -957,10 +957,10 @@
         <v>42185</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.0071247087726951</v>
+        <v>0.0002461550568429</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.0245044231952045</v>
+        <v>-0.0285035695452963</v>
       </c>
       <c r="E19" s="9" t="n">
         <v>42125</v>
@@ -972,10 +972,10 @@
         <v>42216</v>
       </c>
       <c r="B20" t="n">
-        <v>0.0362841901551112</v>
+        <v>0.0255436659490007</v>
       </c>
       <c r="C20" t="n">
-        <v>-0.005767258961163</v>
+        <v>-0.0007705367469683</v>
       </c>
       <c r="E20" s="9" t="n">
         <v>42156</v>
@@ -987,10 +987,10 @@
         <v>42247</v>
       </c>
       <c r="B21" t="n">
-        <v>-0.0472147327940783</v>
+        <v>-0.0485796559560306</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.07549531951551471</v>
+        <v>-0.0801949915149073</v>
       </c>
       <c r="E21" s="9" t="n">
         <v>42186</v>
@@ -1002,10 +1002,10 @@
         <v>42277</v>
       </c>
       <c r="B22" t="n">
-        <v>0.0407765990677275</v>
+        <v>0.0501833901765408</v>
       </c>
       <c r="C22" t="n">
-        <v>-0.0530632295876283</v>
+        <v>-0.0546156103216642</v>
       </c>
       <c r="E22" s="9" t="n">
         <v>42217</v>
@@ -1017,10 +1017,10 @@
         <v>42307</v>
       </c>
       <c r="B23" t="n">
-        <v>0.0750256045116007</v>
+        <v>0.090676010479093</v>
       </c>
       <c r="C23" t="n">
-        <v>0.0886699838442485</v>
+        <v>0.08948339042686849</v>
       </c>
       <c r="E23" s="9" t="n">
         <v>42248</v>
@@ -1032,10 +1032,10 @@
         <v>42338</v>
       </c>
       <c r="B24" t="n">
-        <v>-0.0394903519580411</v>
+        <v>-0.0458825196106727</v>
       </c>
       <c r="C24" t="n">
-        <v>-0.0103350477922475</v>
+        <v>-0.0081792480906111</v>
       </c>
       <c r="E24" s="9" t="n">
         <v>42278</v>
@@ -1047,10 +1047,10 @@
         <v>42369</v>
       </c>
       <c r="B25" t="n">
-        <v>0.0602235604219342</v>
+        <v>0.07278896621530601</v>
       </c>
       <c r="C25" t="n">
-        <v>0.0099641843676856</v>
+        <v>0.0113322349147485</v>
       </c>
       <c r="E25" s="9" t="n">
         <v>42309</v>
@@ -1062,10 +1062,10 @@
         <v>42398</v>
       </c>
       <c r="B26" t="n">
-        <v>-0.0401883522945897</v>
+        <v>-0.042772228696849</v>
       </c>
       <c r="C26" t="n">
-        <v>-0.08068535628633509</v>
+        <v>-0.0842809509078675</v>
       </c>
       <c r="E26" s="9" t="n">
         <v>42339</v>
@@ -1077,10 +1077,10 @@
         <v>42429</v>
       </c>
       <c r="B27" t="n">
-        <v>0.0158996618428314</v>
+        <v>0.0152735161954045</v>
       </c>
       <c r="C27" t="n">
-        <v>-0.0135581254727204</v>
+        <v>-0.0267231419463941</v>
       </c>
       <c r="E27" s="9" t="n">
         <v>42370</v>
@@ -1092,10 +1092,10 @@
         <v>42460</v>
       </c>
       <c r="B28" t="n">
-        <v>0.0495512569409307</v>
+        <v>0.0480989901393358</v>
       </c>
       <c r="C28" t="n">
-        <v>0.0686875589112665</v>
+        <v>0.07415778085701941</v>
       </c>
       <c r="E28" s="9" t="n">
         <v>42401</v>
@@ -1107,10 +1107,10 @@
         <v>42489</v>
       </c>
       <c r="B29" t="n">
-        <v>0.0188467333710436</v>
+        <v>0.0185359145856644</v>
       </c>
       <c r="C29" t="n">
-        <v>0.0316511218767039</v>
+        <v>0.0344298458343944</v>
       </c>
       <c r="E29" s="9" t="n">
         <v>42430</v>
@@ -1122,10 +1122,10 @@
         <v>42521</v>
       </c>
       <c r="B30" t="n">
-        <v>0.0029268720371331</v>
+        <v>0.001694711427783</v>
       </c>
       <c r="C30" t="n">
-        <v>-0.0139600690169181</v>
+        <v>-0.0149271577505522</v>
       </c>
       <c r="E30" s="9" t="n">
         <v>42461</v>
@@ -1137,10 +1137,10 @@
         <v>42551</v>
       </c>
       <c r="B31" t="n">
-        <v>0.0158541384114471</v>
+        <v>0.0076184668300425</v>
       </c>
       <c r="C31" t="n">
-        <v>-0.0107078714833797</v>
+        <v>-0.01635436421676</v>
       </c>
       <c r="E31" s="9" t="n">
         <v>42491</v>
@@ -1152,10 +1152,10 @@
         <v>42580</v>
       </c>
       <c r="B32" t="n">
-        <v>0.0541537488726163</v>
+        <v>0.0555259646978643</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0612765845658077</v>
+        <v>0.07153602239309539</v>
       </c>
       <c r="E32" s="9" t="n">
         <v>42522</v>
@@ -1167,10 +1167,10 @@
         <v>42613</v>
       </c>
       <c r="B33" t="n">
-        <v>-0.024079270526214</v>
+        <v>-0.0242737654412347</v>
       </c>
       <c r="C33" t="n">
-        <v>0.0008255420572559</v>
+        <v>1.205308435116813e-05</v>
       </c>
       <c r="E33" s="9" t="n">
         <v>42552</v>
@@ -1182,10 +1182,10 @@
         <v>42643</v>
       </c>
       <c r="B34" t="n">
-        <v>0.0256669696860347</v>
+        <v>0.0269881073139951</v>
       </c>
       <c r="C34" t="n">
-        <v>0.0181536535648113</v>
+        <v>0.0176385425592738</v>
       </c>
       <c r="E34" s="9" t="n">
         <v>42583</v>
@@ -1197,10 +1197,10 @@
         <v>42674</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.0013180637944866</v>
+        <v>-0.0034591226621163</v>
       </c>
       <c r="C35" t="n">
-        <v>0.0021874200449166</v>
+        <v>0.008011040932537</v>
       </c>
       <c r="E35" s="9" t="n">
         <v>42614</v>
@@ -1212,10 +1212,10 @@
         <v>42704</v>
       </c>
       <c r="B36" t="n">
-        <v>-0.0375903651223152</v>
+        <v>-0.0359954698252582</v>
       </c>
       <c r="C36" t="n">
-        <v>-0.0193904334051159</v>
+        <v>-0.0170576029033294</v>
       </c>
       <c r="E36" s="9" t="n">
         <v>42644</v>
@@ -1227,10 +1227,10 @@
         <v>42734</v>
       </c>
       <c r="B37" t="n">
-        <v>-0.014255018075839</v>
+        <v>-0.0097685226147365</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0041856303132661</v>
+        <v>0.006482280129466</v>
       </c>
       <c r="E37" s="9" t="n">
         <v>42675</v>
@@ -1242,10 +1242,10 @@
         <v>42766</v>
       </c>
       <c r="B38" t="n">
-        <v>0.0490613440451728</v>
+        <v>0.0470504590453536</v>
       </c>
       <c r="C38" t="n">
-        <v>0.0440280283249324</v>
+        <v>0.0413581263721802</v>
       </c>
       <c r="E38" s="9" t="n">
         <v>42705</v>
@@ -1257,10 +1257,10 @@
         <v>42794</v>
       </c>
       <c r="B39" t="n">
-        <v>0.0077573797731842</v>
+        <v>0.0068269871339286</v>
       </c>
       <c r="C39" t="n">
-        <v>0.0202206544130379</v>
+        <v>0.0210719845945688</v>
       </c>
       <c r="E39" s="9" t="n">
         <v>42736</v>
@@ -1272,10 +1272,10 @@
         <v>42825</v>
       </c>
       <c r="B40" t="n">
-        <v>0.0184946234971113</v>
+        <v>0.0122173796579062</v>
       </c>
       <c r="C40" t="n">
-        <v>0.0074971345141355</v>
+        <v>0.0077328581774854</v>
       </c>
       <c r="E40" s="9" t="n">
         <v>42767</v>
@@ -1287,10 +1287,10 @@
         <v>42853</v>
       </c>
       <c r="B41" t="n">
-        <v>0.0039226656247632</v>
+        <v>0.0071246012108509</v>
       </c>
       <c r="C41" t="n">
-        <v>0.0069527467047144</v>
+        <v>0.0035853568401641</v>
       </c>
       <c r="E41" s="9" t="n">
         <v>42795</v>
@@ -1302,10 +1302,10 @@
         <v>42886</v>
       </c>
       <c r="B42" t="n">
-        <v>0.0443775644276037</v>
+        <v>0.0472142539360216</v>
       </c>
       <c r="C42" t="n">
-        <v>0.0215623610036581</v>
+        <v>0.0145419646807492</v>
       </c>
       <c r="E42" s="9" t="n">
         <v>42826</v>
@@ -1317,10 +1317,10 @@
         <v>42916</v>
       </c>
       <c r="B43" t="n">
-        <v>0.0021103486769346</v>
+        <v>0.008620478882056099</v>
       </c>
       <c r="C43" t="n">
-        <v>0.0117897180733099</v>
+        <v>0.0134542234637538</v>
       </c>
       <c r="E43" s="9" t="n">
         <v>42856</v>
@@ -1332,10 +1332,10 @@
         <v>42947</v>
       </c>
       <c r="B44" t="n">
-        <v>0.0170563316806201</v>
+        <v>0.0198625289579658</v>
       </c>
       <c r="C44" t="n">
-        <v>0.0291124290491594</v>
+        <v>0.0316703510907277</v>
       </c>
       <c r="E44" s="9" t="n">
         <v>42887</v>
@@ -1347,10 +1347,10 @@
         <v>42978</v>
       </c>
       <c r="B45" t="n">
-        <v>-0.009151411715928299</v>
+        <v>-0.0070545404784581</v>
       </c>
       <c r="C45" t="n">
-        <v>0.0009695412676496001</v>
+        <v>0.0002686130151001</v>
       </c>
       <c r="E45" s="9" t="n">
         <v>42917</v>
@@ -1362,10 +1362,10 @@
         <v>43007</v>
       </c>
       <c r="B46" t="n">
-        <v>-0.0111370478662533</v>
+        <v>-0.008373565963686</v>
       </c>
       <c r="C46" t="n">
-        <v>0.009010002824520601</v>
+        <v>0.0092409725393038</v>
       </c>
       <c r="E46" s="9" t="n">
         <v>42948</v>
@@ -1377,10 +1377,10 @@
         <v>43039</v>
       </c>
       <c r="B47" t="n">
-        <v>0.0196873112697769</v>
+        <v>0.020358541013542</v>
       </c>
       <c r="C47" t="n">
-        <v>0.0359279854803487</v>
+        <v>0.0338737002409235</v>
       </c>
       <c r="E47" s="9" t="n">
         <v>42979</v>
@@ -1392,10 +1392,10 @@
         <v>43069</v>
       </c>
       <c r="B48" t="n">
-        <v>0.0277792357849402</v>
+        <v>0.0287937302851727</v>
       </c>
       <c r="C48" t="n">
-        <v>0.0242737538807348</v>
+        <v>0.0222537618704587</v>
       </c>
       <c r="E48" s="9" t="n">
         <v>43009</v>
@@ -1407,10 +1407,10 @@
         <v>43098</v>
       </c>
       <c r="B49" t="n">
-        <v>-0.0097551979958664</v>
+        <v>-0.0010932106798448</v>
       </c>
       <c r="C49" t="n">
-        <v>0.0111202132151878</v>
+        <v>0.0161871601657242</v>
       </c>
       <c r="E49" s="9" t="n">
         <v>43040</v>
@@ -1422,10 +1422,10 @@
         <v>43131</v>
       </c>
       <c r="B50" t="n">
-        <v>0.0324951451065878</v>
+        <v>0.0318115378978583</v>
       </c>
       <c r="C50" t="n">
-        <v>0.0475087345593656</v>
+        <v>0.0438933515081785</v>
       </c>
       <c r="E50" s="9" t="n">
         <v>43070</v>
@@ -1437,10 +1437,10 @@
         <v>43159</v>
       </c>
       <c r="B51" t="n">
-        <v>-0.0136683878850766</v>
+        <v>-0.0182930069181143</v>
       </c>
       <c r="C51" t="n">
-        <v>-0.022999564396508</v>
+        <v>-0.025278348843201</v>
       </c>
       <c r="E51" s="9" t="n">
         <v>43101</v>
@@ -1452,10 +1452,10 @@
         <v>43189</v>
       </c>
       <c r="B52" t="n">
-        <v>-0.0014156455627489</v>
+        <v>-0.0041485021446784</v>
       </c>
       <c r="C52" t="n">
-        <v>-0.0254556263632574</v>
+        <v>-0.0283060471691287</v>
       </c>
       <c r="E52" s="9" t="n">
         <v>43132</v>
@@ -1467,10 +1467,10 @@
         <v>43220</v>
       </c>
       <c r="B53" t="n">
-        <v>0.0008442643548647</v>
+        <v>-0.0022123804015661</v>
       </c>
       <c r="C53" t="n">
-        <v>0.0127323274109773</v>
+        <v>0.0134068486962106</v>
       </c>
       <c r="E53" s="9" t="n">
         <v>43160</v>
@@ -1482,10 +1482,10 @@
         <v>43251</v>
       </c>
       <c r="B54" t="n">
-        <v>-0.0013775519625561</v>
+        <v>-0.0040157251109545</v>
       </c>
       <c r="C54" t="n">
-        <v>-0.0083947435344192</v>
+        <v>-0.008639777072155101</v>
       </c>
       <c r="E54" s="9" t="n">
         <v>43191</v>
@@ -1497,10 +1497,10 @@
         <v>43280</v>
       </c>
       <c r="B55" t="n">
-        <v>-0.0121122899673803</v>
+        <v>-0.0159189899460313</v>
       </c>
       <c r="C55" t="n">
-        <v>-0.022661244433913</v>
+        <v>-0.0171139294279305</v>
       </c>
       <c r="E55" s="9" t="n">
         <v>43221</v>
@@ -1512,10 +1512,10 @@
         <v>43312</v>
       </c>
       <c r="B56" t="n">
-        <v>0.0051946767640506</v>
+        <v>-0.0012628737934474</v>
       </c>
       <c r="C56" t="n">
-        <v>0.0107465930998898</v>
+        <v>0.0139472513290285</v>
       </c>
       <c r="E56" s="9" t="n">
         <v>43252</v>
@@ -1527,10 +1527,10 @@
         <v>43343</v>
       </c>
       <c r="B57" t="n">
-        <v>-0.0014727434172006</v>
+        <v>-0.0063861230676702</v>
       </c>
       <c r="C57" t="n">
-        <v>-0.006414756637926</v>
+        <v>-0.009841112947684199</v>
       </c>
       <c r="E57" s="9" t="n">
         <v>43282</v>
@@ -1542,10 +1542,10 @@
         <v>43371</v>
       </c>
       <c r="B58" t="n">
-        <v>0.0179223587264144</v>
+        <v>0.019790633600766</v>
       </c>
       <c r="C58" t="n">
-        <v>0.0191073189557145</v>
+        <v>0.0174750582802053</v>
       </c>
       <c r="E58" s="9" t="n">
         <v>43313</v>
@@ -1557,10 +1557,10 @@
         <v>43404</v>
       </c>
       <c r="B59" t="n">
-        <v>-0.054838513711146</v>
+        <v>-0.0599083869218941</v>
       </c>
       <c r="C59" t="n">
-        <v>-0.0841284269157723</v>
+        <v>-0.0798797500562282</v>
       </c>
       <c r="E59" s="9" t="n">
         <v>43344</v>
@@ -1572,10 +1572,10 @@
         <v>43434</v>
       </c>
       <c r="B60" t="n">
-        <v>-0.002187665570733</v>
+        <v>0.0058642905499601</v>
       </c>
       <c r="C60" t="n">
-        <v>0.0151763507552339</v>
+        <v>0.010447179975125</v>
       </c>
       <c r="E60" s="9" t="n">
         <v>43374</v>
@@ -1587,10 +1587,10 @@
         <v>43465</v>
       </c>
       <c r="B61" t="n">
-        <v>-0.0143540674099991</v>
+        <v>-0.0175760142761704</v>
       </c>
       <c r="C61" t="n">
-        <v>-0.0506309602993229</v>
+        <v>-0.0474872847379031</v>
       </c>
       <c r="E61" s="9" t="n">
         <v>43405</v>
@@ -1602,10 +1602,10 @@
         <v>43496</v>
       </c>
       <c r="B62" t="n">
-        <v>0.036135231733537</v>
+        <v>0.0435604436707064</v>
       </c>
       <c r="C62" t="n">
-        <v>0.0607248601107742</v>
+        <v>0.0629738787744777</v>
       </c>
       <c r="E62" s="9" t="n">
         <v>43435</v>
@@ -1617,10 +1617,10 @@
         <v>43524</v>
       </c>
       <c r="B63" t="n">
-        <v>-0.0043330393907573</v>
+        <v>-0.0070037462732219</v>
       </c>
       <c r="C63" t="n">
-        <v>0.011955783721321</v>
+        <v>0.0130714198136073</v>
       </c>
       <c r="E63" s="9" t="n">
         <v>43466</v>
@@ -1632,10 +1632,10 @@
         <v>43553</v>
       </c>
       <c r="B64" t="n">
-        <v>-0.0192111803025797</v>
+        <v>-0.0103927205266938</v>
       </c>
       <c r="C64" t="n">
-        <v>0.0109285558175756</v>
+        <v>0.008996699289400599</v>
       </c>
       <c r="E64" s="9" t="n">
         <v>43497</v>
@@ -1647,10 +1647,10 @@
         <v>43585</v>
       </c>
       <c r="B65" t="n">
-        <v>-0.0280489285026653</v>
+        <v>-0.0212132767617696</v>
       </c>
       <c r="C65" t="n">
-        <v>0.0146681314872442</v>
+        <v>0.0143850806574419</v>
       </c>
       <c r="E65" s="9" t="n">
         <v>43525</v>
@@ -1662,10 +1662,10 @@
         <v>43616</v>
       </c>
       <c r="B66" t="n">
-        <v>-0.0273539905738265</v>
+        <v>-0.0249044950171711</v>
       </c>
       <c r="C66" t="n">
-        <v>-0.0390842445388862</v>
+        <v>-0.0376618441688143</v>
       </c>
       <c r="E66" s="9" t="n">
         <v>43556</v>
@@ -1677,10 +1677,10 @@
         <v>43644</v>
       </c>
       <c r="B67" t="n">
-        <v>0.0123629614220318</v>
+        <v>0.0243942341889191</v>
       </c>
       <c r="C67" t="n">
-        <v>0.0439558404804037</v>
+        <v>0.0446590075498522</v>
       </c>
       <c r="E67" s="9" t="n">
         <v>43586</v>
@@ -1692,10 +1692,10 @@
         <v>43677</v>
       </c>
       <c r="B68" t="n">
-        <v>-0.0024646483191007</v>
+        <v>-0.0038718946671578</v>
       </c>
       <c r="C68" t="n">
-        <v>-0.0029648380701892</v>
+        <v>-0.0014780259159512</v>
       </c>
       <c r="E68" s="9" t="n">
         <v>43617</v>
@@ -1707,10 +1707,10 @@
         <v>43707</v>
       </c>
       <c r="B69" t="n">
-        <v>-0.0280017519296128</v>
+        <v>-0.0233458334169784</v>
       </c>
       <c r="C69" t="n">
-        <v>-0.026484400721349</v>
+        <v>-0.0295321958878784</v>
       </c>
       <c r="E69" s="9" t="n">
         <v>43647</v>
@@ -1722,10 +1722,10 @@
         <v>43738</v>
       </c>
       <c r="B70" t="n">
-        <v>0.0284686051457225</v>
+        <v>0.0260494334214674</v>
       </c>
       <c r="C70" t="n">
-        <v>0.029704659620727</v>
+        <v>0.0316967536938187</v>
       </c>
       <c r="E70" s="9" t="n">
         <v>43678</v>
@@ -1737,10 +1737,10 @@
         <v>43769</v>
       </c>
       <c r="B71" t="n">
-        <v>0.0219925914637798</v>
+        <v>0.02810560895348</v>
       </c>
       <c r="C71" t="n">
-        <v>0.0416171083855398</v>
+        <v>0.0422250301033225</v>
       </c>
       <c r="E71" s="9" t="n">
         <v>43709</v>
@@ -1752,10 +1752,10 @@
         <v>43798</v>
       </c>
       <c r="B72" t="n">
-        <v>-7.001846893496123e-05</v>
+        <v>-0.0034201862545937</v>
       </c>
       <c r="C72" t="n">
-        <v>0.0016869720522591</v>
+        <v>0.000662339655688</v>
       </c>
       <c r="E72" s="9" t="n">
         <v>43739</v>
@@ -1767,10 +1767,10 @@
         <v>43830</v>
       </c>
       <c r="B73" t="n">
-        <v>0.0268849732463479</v>
+        <v>0.0239271265582518</v>
       </c>
       <c r="C73" t="n">
-        <v>0.024648829860994</v>
+        <v>0.0265870733014948</v>
       </c>
       <c r="E73" s="9" t="n">
         <v>43770</v>
@@ -1782,10 +1782,10 @@
         <v>43861</v>
       </c>
       <c r="B74" t="n">
-        <v>-0.0237718602131903</v>
+        <v>-0.022748673683341</v>
       </c>
       <c r="C74" t="n">
-        <v>-0.0179598865111262</v>
+        <v>-0.0181437699909169</v>
       </c>
       <c r="E74" s="9" t="n">
         <v>43800</v>
@@ -1797,10 +1797,10 @@
         <v>43889</v>
       </c>
       <c r="B75" t="n">
-        <v>-0.0589729661281852</v>
+        <v>-0.07849270332025569</v>
       </c>
       <c r="C75" t="n">
-        <v>-0.0827545264983742</v>
+        <v>-0.08249361081516091</v>
       </c>
       <c r="E75" s="9" t="n">
         <v>43831</v>
@@ -1812,10 +1812,10 @@
         <v>43921</v>
       </c>
       <c r="B76" t="n">
-        <v>-0.0784991160058835</v>
+        <v>-0.0736254181473973</v>
       </c>
       <c r="C76" t="n">
-        <v>-0.1075897946467893</v>
+        <v>-0.114422511974802</v>
       </c>
       <c r="E76" s="9" t="n">
         <v>43862</v>
@@ -1827,10 +1827,10 @@
         <v>43951</v>
       </c>
       <c r="B77" t="n">
-        <v>0.0692705259174899</v>
+        <v>0.0370015040650085</v>
       </c>
       <c r="C77" t="n">
-        <v>0.0654031263308212</v>
+        <v>0.065716790890928</v>
       </c>
       <c r="E77" s="9" t="n">
         <v>43891</v>
@@ -1842,10 +1842,10 @@
         <v>43980</v>
       </c>
       <c r="B78" t="n">
-        <v>-0.0101542430125601</v>
+        <v>0.005180396009486</v>
       </c>
       <c r="C78" t="n">
-        <v>0.0360976569587131</v>
+        <v>0.0332631188596974</v>
       </c>
       <c r="E78" s="9" t="n">
         <v>43922</v>
@@ -1857,10 +1857,10 @@
         <v>44012</v>
       </c>
       <c r="B79" t="n">
-        <v>-0.0061225733180612</v>
+        <v>-0.00776327042185</v>
       </c>
       <c r="C79" t="n">
-        <v>0.0206342925218138</v>
+        <v>0.0221267154177887</v>
       </c>
       <c r="E79" s="9" t="n">
         <v>43952</v>
@@ -1872,10 +1872,10 @@
         <v>44043</v>
       </c>
       <c r="B80" t="n">
-        <v>-0.008549283008290399</v>
+        <v>-0.0135344617798878</v>
       </c>
       <c r="C80" t="n">
-        <v>-0.0075143424968535</v>
+        <v>-0.0071339507916917</v>
       </c>
       <c r="E80" s="9" t="n">
         <v>43983</v>
@@ -1887,10 +1887,10 @@
         <v>44074</v>
       </c>
       <c r="B81" t="n">
-        <v>0.0381851599550607</v>
+        <v>0.0491490776440052</v>
       </c>
       <c r="C81" t="n">
-        <v>0.0646055240202412</v>
+        <v>0.06659854055011021</v>
       </c>
       <c r="E81" s="9" t="n">
         <v>44013</v>
@@ -1902,10 +1902,10 @@
         <v>44104</v>
       </c>
       <c r="B82" t="n">
-        <v>-0.0187781335998686</v>
+        <v>-0.0216794320972006</v>
       </c>
       <c r="C82" t="n">
-        <v>-0.011691058279204</v>
+        <v>-0.0155821181693188</v>
       </c>
       <c r="E82" s="9" t="n">
         <v>44044</v>
@@ -1917,10 +1917,10 @@
         <v>44134</v>
       </c>
       <c r="B83" t="n">
-        <v>-0.0270284998594713</v>
+        <v>-0.0334684153700058</v>
       </c>
       <c r="C83" t="n">
-        <v>-0.0123324731874683</v>
+        <v>-0.0111471103774918</v>
       </c>
       <c r="E83" s="9" t="n">
         <v>44075</v>
@@ -1932,10 +1932,10 @@
         <v>44165</v>
       </c>
       <c r="B84" t="n">
-        <v>0.0552894543162445</v>
+        <v>0.06680603642057251</v>
       </c>
       <c r="C84" t="n">
-        <v>0.130681155663674</v>
+        <v>0.1329161675884338</v>
       </c>
       <c r="E84" s="9" t="n">
         <v>44105</v>
@@ -1947,10 +1947,10 @@
         <v>44196</v>
       </c>
       <c r="B85" t="n">
-        <v>0.0066955889512044</v>
+        <v>0.0258977349237824</v>
       </c>
       <c r="C85" t="n">
-        <v>0.0444317954232345</v>
+        <v>0.0450716360875853</v>
       </c>
       <c r="E85" s="9" t="n">
         <v>44136</v>
@@ -1962,10 +1962,10 @@
         <v>44225</v>
       </c>
       <c r="B86" t="n">
-        <v>0.0314618326420796</v>
+        <v>0.0230815167694317</v>
       </c>
       <c r="C86" t="n">
-        <v>-0.0048351013302278</v>
+        <v>-0.0043583449855419</v>
       </c>
       <c r="E86" s="9" t="n">
         <v>44166</v>
@@ -1977,10 +1977,10 @@
         <v>44253</v>
       </c>
       <c r="B87" t="n">
-        <v>-0.0170230997504482</v>
+        <v>-0.0147355996353388</v>
       </c>
       <c r="C87" t="n">
-        <v>0.0232990132743903</v>
+        <v>0.0297289332374099</v>
       </c>
       <c r="E87" s="9" t="n">
         <v>44197</v>
@@ -1992,10 +1992,10 @@
         <v>44286</v>
       </c>
       <c r="B88" t="n">
-        <v>0.0287623113524269</v>
+        <v>0.0343605325172211</v>
       </c>
       <c r="C88" t="n">
-        <v>0.0153935873574069</v>
+        <v>0.0149058555454091</v>
       </c>
       <c r="E88" s="9" t="n">
         <v>44228</v>
@@ -2007,10 +2007,10 @@
         <v>44316</v>
       </c>
       <c r="B89" t="n">
-        <v>-0.0024991770919677</v>
+        <v>-0.0085769411553223</v>
       </c>
       <c r="C89" t="n">
-        <v>-0.0007648688726008</v>
+        <v>-0.0020975648486187</v>
       </c>
       <c r="E89" s="9" t="n">
         <v>44256</v>
@@ -2022,10 +2022,10 @@
         <v>44347</v>
       </c>
       <c r="B90" t="n">
-        <v>0.0132933222736635</v>
+        <v>0.0075771297951094</v>
       </c>
       <c r="C90" t="n">
-        <v>0.0209556919666648</v>
+        <v>0.021772731935455</v>
       </c>
       <c r="E90" s="9" t="n">
         <v>44287</v>
@@ -2037,10 +2037,10 @@
         <v>44377</v>
       </c>
       <c r="B91" t="n">
-        <v>-0.0007642147858891</v>
+        <v>0.0049625517374662</v>
       </c>
       <c r="C91" t="n">
-        <v>-0.008607642719922299</v>
+        <v>-0.009546970987800101</v>
       </c>
       <c r="E91" s="9" t="n">
         <v>44317</v>
@@ -2052,10 +2052,10 @@
         <v>44407</v>
       </c>
       <c r="B92" t="n">
-        <v>0.0060275862763568</v>
+        <v>-0.0060383292498267</v>
       </c>
       <c r="C92" t="n">
-        <v>-0.0163879310489994</v>
+        <v>-0.0186540335787189</v>
       </c>
       <c r="E92" s="9" t="n">
         <v>44348</v>
@@ -2067,10 +2067,10 @@
         <v>44439</v>
       </c>
       <c r="B93" t="n">
-        <v>0.0218596291197615</v>
+        <v>0.0357850861538765</v>
       </c>
       <c r="C93" t="n">
-        <v>0.0235472672692028</v>
+        <v>0.0235159647373875</v>
       </c>
       <c r="E93" s="9" t="n">
         <v>44378</v>
@@ -2082,10 +2082,10 @@
         <v>44469</v>
       </c>
       <c r="B94" t="n">
-        <v>0.0121218903641477</v>
+        <v>0.0157483532983796</v>
       </c>
       <c r="C94" t="n">
-        <v>0.0108641614297038</v>
+        <v>0.0120222813742093</v>
       </c>
       <c r="E94" s="9" t="n">
         <v>44409</v>
@@ -2097,10 +2097,10 @@
         <v>44498</v>
       </c>
       <c r="B95" t="n">
-        <v>-0.0076368904460683</v>
+        <v>-0.0111591204253823</v>
       </c>
       <c r="C95" t="n">
-        <v>-0.0111454861585684</v>
+        <v>-0.0119290789372227</v>
       </c>
       <c r="E95" s="9" t="n">
         <v>44440</v>
@@ -2112,10 +2112,10 @@
         <v>44530</v>
       </c>
       <c r="B96" t="n">
-        <v>-0.010420070984226</v>
+        <v>-0.0248691732562638</v>
       </c>
       <c r="C96" t="n">
-        <v>-0.0356982050721316</v>
+        <v>-0.0382479160743059</v>
       </c>
       <c r="E96" s="9" t="n">
         <v>44470</v>
@@ -2127,10 +2127,10 @@
         <v>44561</v>
       </c>
       <c r="B97" t="n">
-        <v>0.0146540895698679</v>
+        <v>0.0117617700858736</v>
       </c>
       <c r="C97" t="n">
-        <v>0.028328195448495</v>
+        <v>0.0294420954468159</v>
       </c>
       <c r="E97" s="9" t="n">
         <v>44501</v>
@@ -2142,10 +2142,10 @@
         <v>44592</v>
       </c>
       <c r="B98" t="n">
-        <v>-0.0142503911262826</v>
+        <v>-0.0093915533983738</v>
       </c>
       <c r="C98" t="n">
-        <v>-0.036800243514807</v>
+        <v>-0.0337504427150578</v>
       </c>
       <c r="E98" s="9" t="n">
         <v>44531</v>
@@ -2157,10 +2157,10 @@
         <v>44620</v>
       </c>
       <c r="B99" t="n">
-        <v>0.0199670118068595</v>
+        <v>0.0171992892548055</v>
       </c>
       <c r="C99" t="n">
-        <v>0.0011377458853106</v>
+        <v>0.0021500976971975</v>
       </c>
       <c r="E99" s="9" t="n">
         <v>44562</v>
@@ -2172,10 +2172,10 @@
         <v>44651</v>
       </c>
       <c r="B100" t="n">
-        <v>-0.0339305708209424</v>
+        <v>-0.027930855075548</v>
       </c>
       <c r="C100" t="n">
-        <v>0.015783214618301</v>
+        <v>0.0166491136726589</v>
       </c>
       <c r="E100" s="9" t="n">
         <v>44593</v>
@@ -2187,10 +2187,10 @@
         <v>44680</v>
       </c>
       <c r="B101" t="n">
-        <v>-0.0273126207578517</v>
+        <v>-0.0318420608100496</v>
       </c>
       <c r="C101" t="n">
-        <v>-0.0677131276168874</v>
+        <v>-0.0678887255158839</v>
       </c>
       <c r="E101" s="9" t="n">
         <v>44621</v>
@@ -2202,10 +2202,10 @@
         <v>44712</v>
       </c>
       <c r="B102" t="n">
-        <v>0.0385035338181791</v>
+        <v>0.0233799320798172</v>
       </c>
       <c r="C102" t="n">
-        <v>0.00698188673958</v>
+        <v>0.0073661365847654</v>
       </c>
       <c r="E102" s="9" t="n">
         <v>44652</v>
@@ -2217,10 +2217,10 @@
         <v>44742</v>
       </c>
       <c r="B103" t="n">
-        <v>-0.06324777124982429</v>
+        <v>-0.0466299805463538</v>
       </c>
       <c r="C103" t="n">
-        <v>-0.0714494434963429</v>
+        <v>-0.0714001933577616</v>
       </c>
       <c r="E103" s="9" t="n">
         <v>44682</v>
@@ -2232,10 +2232,10 @@
         <v>44771</v>
       </c>
       <c r="B104" t="n">
-        <v>0.0331656275092946</v>
+        <v>0.0270765204905426</v>
       </c>
       <c r="C104" t="n">
-        <v>0.0432374307202487</v>
+        <v>0.0421750372004175</v>
       </c>
       <c r="E104" s="9" t="n">
         <v>44713</v>
@@ -2247,10 +2247,10 @@
         <v>44804</v>
       </c>
       <c r="B105" t="n">
-        <v>-0.0050043110185632</v>
+        <v>-0.0140285017550387</v>
       </c>
       <c r="C105" t="n">
-        <v>-0.0199187084572835</v>
+        <v>-0.0206299910368805</v>
       </c>
       <c r="E105" s="9" t="n">
         <v>44743</v>
@@ -2262,10 +2262,10 @@
         <v>44834</v>
       </c>
       <c r="B106" t="n">
-        <v>-0.0573195286108208</v>
+        <v>-0.0607103700601502</v>
       </c>
       <c r="C106" t="n">
-        <v>-0.09872846341438581</v>
+        <v>-0.1006793014448188</v>
       </c>
       <c r="E106" s="9" t="n">
         <v>44774</v>
@@ -2277,10 +2277,10 @@
         <v>44865</v>
       </c>
       <c r="B107" t="n">
-        <v>-0.0206592802596433</v>
+        <v>-0.0163774918872795</v>
       </c>
       <c r="C107" t="n">
-        <v>0.0154537207239235</v>
+        <v>0.0136767007551921</v>
       </c>
       <c r="E107" s="9" t="n">
         <v>44805</v>
@@ -2292,10 +2292,10 @@
         <v>44895</v>
       </c>
       <c r="B108" t="n">
-        <v>0.09832976236810401</v>
+        <v>0.1045673974044797</v>
       </c>
       <c r="C108" t="n">
-        <v>0.1065378940390857</v>
+        <v>0.1090450352689806</v>
       </c>
       <c r="E108" s="9" t="n">
         <v>44835</v>
@@ -2307,10 +2307,10 @@
         <v>44925</v>
       </c>
       <c r="B109" t="n">
-        <v>-0.0207041830828527</v>
+        <v>-0.0082180588056305</v>
       </c>
       <c r="C109" t="n">
-        <v>0.0017703432683412</v>
+        <v>0.0017886561636655</v>
       </c>
       <c r="E109" s="9" t="n">
         <v>44866</v>
@@ -2322,10 +2322,10 @@
         <v>44957</v>
       </c>
       <c r="B110" t="n">
-        <v>0.0366481462130185</v>
+        <v>0.0410995849060746</v>
       </c>
       <c r="C110" t="n">
-        <v>0.0652011522005241</v>
+        <v>0.0647740425149352</v>
       </c>
       <c r="E110" s="9" t="n">
         <v>44896</v>
@@ -2337,10 +2337,10 @@
         <v>44985</v>
       </c>
       <c r="B111" t="n">
-        <v>-0.0465416688530787</v>
+        <v>-0.0397469194294353</v>
       </c>
       <c r="C111" t="n">
-        <v>-0.0444018309931057</v>
+        <v>-0.0450509034846863</v>
       </c>
       <c r="E111" s="9" t="n">
         <v>44927</v>
@@ -2352,10 +2352,10 @@
         <v>45016</v>
       </c>
       <c r="B112" t="n">
-        <v>0.0524165648594865</v>
+        <v>0.0406936273895173</v>
       </c>
       <c r="C112" t="n">
-        <v>0.0286049442421165</v>
+        <v>0.0269399978347537</v>
       </c>
       <c r="E112" s="9" t="n">
         <v>44958</v>
@@ -2367,10 +2367,10 @@
         <v>45044</v>
       </c>
       <c r="B113" t="n">
-        <v>0.036151243358694</v>
+        <v>0.0289436621395879</v>
       </c>
       <c r="C113" t="n">
-        <v>0.0066046066365428</v>
+        <v>0.0080365094592743</v>
       </c>
       <c r="E113" s="9" t="n">
         <v>44986</v>
@@ -2382,10 +2382,10 @@
         <v>45077</v>
       </c>
       <c r="B114" t="n">
-        <v>-0.0046519504794748</v>
+        <v>-0.0061349016293079</v>
       </c>
       <c r="C114" t="n">
-        <v>-0.0083835386947808</v>
+        <v>-0.0100691848218455</v>
       </c>
       <c r="E114" s="9" t="n">
         <v>45017</v>
@@ -2397,10 +2397,10 @@
         <v>45107</v>
       </c>
       <c r="B115" t="n">
-        <v>0.0194552289981887</v>
+        <v>0.01915957281711</v>
       </c>
       <c r="C115" t="n">
-        <v>0.0430608879801947</v>
+        <v>0.0459439228596519</v>
       </c>
       <c r="E115" s="9" t="n">
         <v>45047</v>
@@ -2412,10 +2412,10 @@
         <v>45138</v>
       </c>
       <c r="B116" t="n">
-        <v>0.0338357850074215</v>
+        <v>0.0340608623295032</v>
       </c>
       <c r="C116" t="n">
-        <v>0.0351737329093065</v>
+        <v>0.0378259498653461</v>
       </c>
       <c r="E116" s="9" t="n">
         <v>45078</v>
@@ -2427,10 +2427,10 @@
         <v>45169</v>
       </c>
       <c r="B117" t="n">
-        <v>0.0272175115272867</v>
+        <v>0.0067208450783503</v>
       </c>
       <c r="C117" t="n">
-        <v>-0.0317019609414933</v>
+        <v>-0.0315072933862256</v>
       </c>
       <c r="E117" s="9" t="n">
         <v>45108</v>
@@ -2442,10 +2442,10 @@
         <v>45198</v>
       </c>
       <c r="B118" t="n">
-        <v>-0.0144338548124589</v>
+        <v>-0.0127997392867211</v>
       </c>
       <c r="C118" t="n">
-        <v>-0.0188549082307113</v>
+        <v>-0.0172489999182926</v>
       </c>
       <c r="E118" s="9" t="n">
         <v>45139</v>
@@ -2457,10 +2457,10 @@
         <v>45230</v>
       </c>
       <c r="B119" t="n">
-        <v>-0.0289538287806094</v>
+        <v>-0.0203740832487482</v>
       </c>
       <c r="C119" t="n">
-        <v>-0.0459503631595632</v>
+        <v>-0.0480901573243866</v>
       </c>
       <c r="E119" s="9" t="n">
         <v>45170</v>
@@ -2472,10 +2472,10 @@
         <v>45260</v>
       </c>
       <c r="B120" t="n">
-        <v>0.0336368941465958</v>
+        <v>0.044300293004788</v>
       </c>
       <c r="C120" t="n">
-        <v>0.0679908187858861</v>
+        <v>0.06836402533350359</v>
       </c>
       <c r="E120" s="9" t="n">
         <v>45200</v>
@@ -2487,10 +2487,10 @@
         <v>45289</v>
       </c>
       <c r="B121" t="n">
-        <v>-0.1242717964152482</v>
+        <v>-0.0472993985810409</v>
       </c>
       <c r="C121" t="n">
-        <v>0.0491429755217619</v>
+        <v>0.0503942308328531</v>
       </c>
       <c r="E121" s="9" t="n">
         <v>45231</v>
@@ -2502,10 +2502,10 @@
         <v>45322</v>
       </c>
       <c r="B122" t="n">
-        <v>0.0130471225033452</v>
+        <v>0.0151384020965921</v>
       </c>
       <c r="C122" t="n">
-        <v>0.0218027618818123</v>
+        <v>0.0218687773070684</v>
       </c>
       <c r="E122" s="9" t="n">
         <v>45261</v>
@@ -2517,10 +2517,10 @@
         <v>45351</v>
       </c>
       <c r="B123" t="n">
-        <v>0.0020729144706552</v>
+        <v>-0.0006335115255571</v>
       </c>
       <c r="C123" t="n">
-        <v>0.0264554865603872</v>
+        <v>0.0272624412610992</v>
       </c>
       <c r="E123" s="9" t="n">
         <v>45292</v>
@@ -2532,10 +2532,10 @@
         <v>45380</v>
       </c>
       <c r="B124" t="n">
-        <v>0.0448870396945253</v>
+        <v>0.0389025119355257</v>
       </c>
       <c r="C124" t="n">
-        <v>0.0241365225357864</v>
+        <v>0.0252620062438797</v>
       </c>
       <c r="E124" s="9" t="n">
         <v>45323</v>
@@ -2547,10 +2547,10 @@
         <v>45412</v>
       </c>
       <c r="B125" t="n">
-        <v>-0.0180438309815904</v>
+        <v>-0.0181981047761095</v>
       </c>
       <c r="C125" t="n">
-        <v>-0.034066183159725</v>
+        <v>-0.0347744059315882</v>
       </c>
       <c r="E125" s="9" t="n">
         <v>45352</v>
@@ -2562,10 +2562,10 @@
         <v>45443</v>
       </c>
       <c r="B126" t="n">
-        <v>0.0075019773350089</v>
+        <v>-0.0069272074784862</v>
       </c>
       <c r="C126" t="n">
-        <v>0.0116213163305105</v>
+        <v>0.0119565133632475</v>
       </c>
       <c r="E126" s="9" t="n">
         <v>45383</v>
@@ -2577,10 +2577,10 @@
         <v>45471</v>
       </c>
       <c r="B127" t="n">
-        <v>-0.0390905218988838</v>
+        <v>-0.0347753355517561</v>
       </c>
       <c r="C127" t="n">
-        <v>-0.0054189705070492</v>
+        <v>-0.0046919640756411</v>
       </c>
       <c r="E127" s="9" t="n">
         <v>45413</v>
@@ -2592,10 +2592,10 @@
         <v>45504</v>
       </c>
       <c r="B128" t="n">
-        <v>0.0778920321283479</v>
+        <v>0.0608156114374007</v>
       </c>
       <c r="C128" t="n">
-        <v>0.0465302769809573</v>
+        <v>0.0468270012852846</v>
       </c>
       <c r="E128" s="9" t="n">
         <v>45444</v>
@@ -2607,10 +2607,10 @@
         <v>45534</v>
       </c>
       <c r="B129" t="n">
-        <v>-0.0017331985613987</v>
+        <v>0.00827010610081</v>
       </c>
       <c r="C129" t="n">
-        <v>0.0146937501815359</v>
+        <v>0.0141556407471661</v>
       </c>
       <c r="E129" s="9" t="n">
         <v>45474</v>
@@ -2622,10 +2622,10 @@
         <v>45565</v>
       </c>
       <c r="B130" t="n">
-        <v>0.0107595278656082</v>
+        <v>0.0122805137907108</v>
       </c>
       <c r="C130" t="n">
-        <v>0.0199865103985881</v>
+        <v>0.0204298387475872</v>
       </c>
       <c r="E130" s="9" t="n">
         <v>45505</v>
@@ -2637,10 +2637,10 @@
         <v>45596</v>
       </c>
       <c r="B131" t="n">
-        <v>-0.0360610119585291</v>
+        <v>-0.0363201053148279</v>
       </c>
       <c r="C131" t="n">
-        <v>-0.0433874636762671</v>
+        <v>-0.0438711667623903</v>
       </c>
       <c r="E131" s="9" t="n">
         <v>45536</v>
@@ -2652,10 +2652,10 @@
         <v>45625</v>
       </c>
       <c r="B132" t="n">
-        <v>0.0450887400567218</v>
+        <v>0.0318679318594734</v>
       </c>
       <c r="C132" t="n">
-        <v>0.0047776943894237</v>
+        <v>0.0031871728545217</v>
       </c>
       <c r="E132" s="9" t="n">
         <v>45566</v>
@@ -2667,10 +2667,10 @@
         <v>45657</v>
       </c>
       <c r="B133" t="n">
-        <v>-0.0200379823311739</v>
+        <v>-0.0163869093303216</v>
       </c>
       <c r="C133" t="n">
-        <v>-0.010902292498802</v>
+        <v>-0.0098691156983703</v>
       </c>
       <c r="E133" s="9" t="n">
         <v>45597</v>
@@ -2682,10 +2682,10 @@
         <v>45688</v>
       </c>
       <c r="B134" t="n">
-        <v>0.04297859373411</v>
+        <v>0.0254325769262944</v>
       </c>
       <c r="C134" t="n">
-        <v>0.016228420056879</v>
+        <v>0.0147391209479191</v>
       </c>
       <c r="E134" s="9" t="n">
         <v>45627</v>
@@ -2697,10 +2697,10 @@
         <v>45716</v>
       </c>
       <c r="B135" t="n">
-        <v>0.0489264912281381</v>
+        <v>0.0335947760325025</v>
       </c>
       <c r="C135" t="n">
-        <v>-0.0092809624762774</v>
+        <v>-0.008830818505325</v>
       </c>
       <c r="E135" s="9" t="n">
         <v>45658</v>
@@ -2712,10 +2712,10 @@
         <v>45747</v>
       </c>
       <c r="B136" t="n">
-        <v>0.0373980583438695</v>
+        <v>0.0331071496039094</v>
       </c>
       <c r="C136" t="n">
-        <v>0.0042191259708773</v>
+        <v>0.0040357097411973</v>
       </c>
       <c r="E136" s="9" t="n">
         <v>45689</v>
@@ -2727,10 +2727,10 @@
         <v>45777</v>
       </c>
       <c r="B137" t="n">
-        <v>0.0749363207391939</v>
+        <v>0.0658549106856807</v>
       </c>
       <c r="C137" t="n">
-        <v>0.0537093125195659</v>
+        <v>0.0550897281260333</v>
       </c>
       <c r="E137" s="9" t="n">
         <v>45717</v>
@@ -2742,10 +2742,10 @@
         <v>45807</v>
       </c>
       <c r="B138" t="n">
-        <v>0.0184678385216009</v>
+        <v>0.0237888738885093</v>
       </c>
       <c r="C138" t="n">
-        <v>0.0382922269183745</v>
+        <v>0.0386891516634081</v>
       </c>
       <c r="E138" s="9" t="n">
         <v>45748</v>
@@ -2757,10 +2757,10 @@
         <v>45838</v>
       </c>
       <c r="B139" t="n">
-        <v>0.0477679742690069</v>
+        <v>0.0358068869139919</v>
       </c>
       <c r="C139" t="n">
-        <v>0.021670640724601</v>
+        <v>0.0228626694842976</v>
       </c>
       <c r="E139" s="9" t="n">
         <v>45778</v>
@@ -2772,10 +2772,10 @@
         <v>45869</v>
       </c>
       <c r="B140" t="n">
-        <v>0.012694939976014</v>
+        <v>0.0131448751835017</v>
       </c>
       <c r="C140" t="n">
-        <v>-0.0015308589915159</v>
+        <v>-0.0002123242528831</v>
       </c>
       <c r="E140" s="9" t="n">
         <v>45809</v>
@@ -2787,10 +2787,10 @@
         <v>45898</v>
       </c>
       <c r="B141" t="n">
-        <v>0.0354718118732805</v>
+        <v>0.0459601424531922</v>
       </c>
       <c r="C141" t="n">
-        <v>0.0614456168602271</v>
+        <v>0.0616995332510839</v>
       </c>
       <c r="E141" s="9" t="n">
         <v>45839</v>
@@ -2802,10 +2802,10 @@
         <v>45930</v>
       </c>
       <c r="B142" t="n">
-        <v>0.021533670028697</v>
+        <v>0.0177640203376163</v>
       </c>
       <c r="C142" t="n">
-        <v>0.0149629020739231</v>
+        <v>0.0153728424977929</v>
       </c>
       <c r="E142" s="9" t="n">
         <v>45870</v>
@@ -2817,10 +2817,10 @@
         <v>45961</v>
       </c>
       <c r="B143" t="n">
-        <v>-0.0016377407785709</v>
+        <v>-0.000176972296396</v>
       </c>
       <c r="C143" t="n">
-        <v>0.0265252726536321</v>
+        <v>0.0284469698425511</v>
       </c>
       <c r="E143" s="9" t="n">
         <v>45901</v>
@@ -2832,10 +2832,10 @@
         <v>45989</v>
       </c>
       <c r="B144" t="n">
-        <v>0.0259214143527395</v>
+        <v>0.0234809853763016</v>
       </c>
       <c r="C144" t="n">
-        <v>-0.0067052829911501</v>
+        <v>-0.0064464000436423</v>
       </c>
       <c r="E144" s="9" t="n">
         <v>45931</v>
@@ -2847,10 +2847,10 @@
         <v>46022</v>
       </c>
       <c r="B145" t="n">
-        <v>-0.0022332187009084</v>
+        <v>-0.0042499103357053</v>
       </c>
       <c r="C145" t="n">
-        <v>0.0076617247707648</v>
+        <v>0.0073398326941541</v>
       </c>
       <c r="E145" s="9" t="n">
         <v>45962</v>

</xml_diff>